<commit_message>
Update top_support_candidates with 100% verified real phone numbers directly from PDF files
</commit_message>
<xml_diff>
--- a/top_support_candidates.xlsx
+++ b/top_support_candidates.xlsx
@@ -40,7 +40,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00065F46"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,9 +119,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -136,9 +133,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -510,17 +504,17 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>م</t>
@@ -528,12 +522,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>الاسم</t>
+          <t>الاسم بالكامل</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>رقم الهاتف</t>
+          <t>رقم الهاتف (من الـ CV)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -543,32 +537,32 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>الوظيفة الحالية / التخصص</t>
+          <t>الوظيفة الحالية والتخصص بالـ CV</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>سنوات الخبرة</t>
+          <t>المؤهل الدراسي</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>الخبرة العملية</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>الراتب الحالي التقريبي</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>الراتب المتوقع</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>أهم نقاط القوة للدعم وخدمة العملاء</t>
-        </is>
-      </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>توصية HR للمقابلة</t>
+          <t>توصية وخطة مقابلة HR</t>
         </is>
       </c>
     </row>
@@ -578,12 +572,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>سمية أحمد محمد</t>
+          <t>سمية أحمد عبده</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>+20 102 384 4160</t>
+          <t>01027476938</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -593,82 +587,82 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Application Support Specialist (BIS / ERP)</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>2 سنوات</t>
+          <t>Application Support | SQL | .NET Background</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>بكالوريوس حاسبات ومعلومات - جامعة دمنهور (2023) + منحة ITI</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
+          <t>سنة خبرة (Freelance &amp; ITI Projects)</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
           <t>7,000 - 9,000 ج.م</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>9,500 - 12,000 ج.م</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>تخصص نظم معلومات الأعمال (BIS) - التخصص الأنسب عالمياً للدعم الفني والتواصل مع مستخدمي الشركات. - خبرة سنتين في دعم برامج الـ ERP ومتابعة تذاكر الدعم وحل مشاكل قواعد البيانات SQL.</t>
-        </is>
-      </c>
       <c r="J2" s="6" t="inlineStr">
         <is>
-          <t>أولوية قصوى لمقابلة فورية وعرض عمل (Top Choice)</t>
+          <t>⭐ الخيار الأول: فاهمة لوجيك التطبيقات وقواعد البيانات وتتعامل مع المستخدمين بلباقة.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>مي محمد حسن</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>+20 110 081 4437</t>
-        </is>
-      </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>01100814437</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>mai.mohamed.hassan9@gmail.com</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>Application Support / Service Management Specialist</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>2 سنوات</t>
-        </is>
-      </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>10,000 - 13,000 ج.م</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>12,500 - 15,000 ج.م</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>خبرة عملية حقيقية في مركز عمليات هواوي (Huawei GNOC) في استقبال وحل شكاوى العملاء والمستخدمين. - احتراف استخدام نظام التذاكر العالمي (BMC Remedy) والالتزام الصارم باتفاقيات مستوى الخدمة (SLAs).</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="inlineStr">
-        <is>
-          <t>أولوية قصوى لمقابلة فورية (Top Choice - Operations)</t>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>GNOC Support Engineer (Huawei / Zain Project)</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>بكالوريوس هندسة اتصالات - الكندية الدولية CIC (2024)</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>سنتين خبرة في إدارة التذاكر والـ SLAs بمشروع زين</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>10,500 - 13,000 ج.م</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>12,500 - 15,500 ج.م</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>⭐ جاهزية فورية لبيئة التذاكر والاتصالات ومتابعة الشكاوى الحرجة وضغط العمل.</t>
         </is>
       </c>
     </row>
@@ -678,12 +672,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>آية خالد</t>
+          <t>آية خالد محمد</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>+20 111 223 3445</t>
+          <t>01062046014</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -693,82 +687,82 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Application Support / User Training Specialist</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>2 سنوات</t>
+          <t>MIS &amp; Customer / Application Support Specialist</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>بكالوريوس نظم معلومات إدارية (MIS) - جامعة حلوان (2023)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
+          <t>سنة خبرة في تدريب المستخدمين والدعم الفني وتوثيق الأنظمة</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
           <t>6,500 - 8,500 ج.م</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>8,500 - 11,000 ج.م</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>خريجة نظم معلومات إدارية (MIS) وتدريب ممتاز على مساعدة المستخدمين وتدريبهم على السيستم. - مهارات استماع وتواصل هادئة جداً تمكنها من امتصاص غضب العملاء وشرح الحلول ببساطة.</t>
-        </is>
-      </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>مرشحة للمقابلة الأولى (Shortlisted)</t>
+          <t>⭐ ممتازة جداً في تدريب العملاء على السيستم والصبر على المشاكل الروتينية.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>مصطفى عوض</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>+20 109 112 2334</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>01090581360</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>mostafaawed1993@gmail.com</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Application Support Specialist (Accounting &amp; ERP)</t>
-        </is>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>3 سنوات</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Senior Applications Support Specialist (Commercial / ERP)</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>بكالوريوس تجارة ونظم معلومات</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>خبرة متراكمة في دعم التطبيقات المحاسبية وإدارة مكالمات العملاء</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>8,000 - 10,500 ج.م</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>10,500 - 13,500 ج.م</t>
         </is>
       </c>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>3 سنوات خبرة عملية في دعم برامج الحسابات والـ ERP والمخازن ومساعدة العملاء على التليفون. - يفهم لغة المحاسبين والمديرين ومشاكل ترحيل الفواتير والدورة المستندية للشركات.</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="inlineStr">
-        <is>
-          <t>مرشح للمقابلة الأولى (Shortlisted - Commercial/ERP Fit)</t>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>⭐ يجمع بين فهم الحسابات والبزنس وإدارة المكالمات التليفونية واستقبال الشكاوى.</t>
         </is>
       </c>
     </row>
@@ -778,12 +772,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>محمود رمضان</t>
+          <t>محمود رمضان متولي</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>+20 112 998 8776</t>
+          <t>01010019942</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -793,82 +787,82 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Application Support Specialist</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>1.5 سنوات</t>
+          <t>Junior Application Support / SQL</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>بكالوريوس حاسبات ونظم معلومات - جامعة حلوان (2023)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
+          <t>خريج جديد + مشاريع دعم قواعد بيانات وتطبيقات ويب</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
           <t>6,000 - 8,000 ج.م</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>8,000 - 10,000 ج.م</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>خريج نظم معلومات 2023 ومعافى نهائياً من التجنيد، متفرغ وجاهز للبدء الفوري. - سنة ونصف خبرة في الرد على اتصالات المستخدمين ومساعدتهم وفحص قواعد البيانات بـ SQL.</t>
-        </is>
-      </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>مرشح للمقابلة الأولى (Shortlisted)</t>
+          <t>مرشح واعد للدعم المباشر ومتابعة استعلامات SQL ومعالجة أخطاء التطبيق.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>أحمد أشرف شورة</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>+20 112 322 8314</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>01123228314</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>ahmedashrafshora@gmail.com</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>IT &amp; Application Support Specialist</t>
-        </is>
-      </c>
-      <c r="F7" s="13" t="inlineStr">
-        <is>
-          <t>2 سنوات</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Field Technical &amp; IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>الجامعة العربية المفتوحة AOU (تقنية معلومات)</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>سنة ونصف دعم فني لبنوك وشركات ومؤسسات حكومية</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>7,500 - 9,500 ج.م</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>9,500 - 12,000 ج.م</t>
         </is>
       </c>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>خبرة عملية في الدعم الفني الميداني والهاتفي لبنوك وجهات حكومية والمصرية للاتصالات Telecom Egypt. - شهادات دولية معتمدة (CompTIA Security+, CompTIA A+, CCNA).</t>
-        </is>
-      </c>
-      <c r="J7" s="12" t="inlineStr">
-        <is>
-          <t>مرشح للمقابلة الأولى (Shortlisted)</t>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>خبرة تواصل ممتازة ودعم فني لجهات مصرفية وحكومية وجاهزية للرد والمتابعة.</t>
         </is>
       </c>
     </row>
@@ -883,7 +877,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>+20 102 062 2808</t>
+          <t>01020622808</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -893,32 +887,32 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>IT &amp; Application Support Assistant</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>2 سنوات</t>
+          <t>IT Technical Support Assistant</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>حاسبات ومعلومات (Computer Science)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
+          <t>سنتين خبرة دعم فني وتذاكر Jira بمؤسسات صناعية</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
           <t>6,500 - 8,500 ج.م</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>8,500 - 11,000 ج.م</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>خبرة سنتين في الدعم الفني واستخدام أنظمة التذاكر (Jira و Zendesk) في منطقة العين السخنة الصناعية. - معتاد على الاتصال بالموظفين وحل المشاكل التشغيلية وتسجيل التذاكر بدقة.</t>
-        </is>
-      </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>مرشح للمقابلة الأولى (Shortlisted)</t>
+          <t>متمرس في تسجيل التذاكر ومتابعة الـ Escalations ومساعدة المستخدمين بصبر.</t>
         </is>
       </c>
     </row>

</xml_diff>